<commit_message>
Removed wrong Gallium intensity for c-Si.
</commit_message>
<xml_diff>
--- a/premise/data/metals/SI_2_Material_requirements.xlsx
+++ b/premise/data/metals/SI_2_Material_requirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hahnme_a\PycharmProjects\premise\premise\data\metals\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davidba\LCA\scenarioLCA\premise_metals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F4ACDE-74C1-440C-B5EA-5E68E6F44D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67D79D8-2156-425C-A660-B36663FF2295}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14355" yWindow="-16200" windowWidth="14610" windowHeight="15585" tabRatio="602" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14355" yWindow="-16200" windowWidth="14610" windowHeight="15585" tabRatio="602" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Materials" sheetId="1" r:id="rId1"/>
@@ -40,23 +40,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1416" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="393">
   <si>
     <t>DLR</t>
   </si>
@@ -11383,7 +11372,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B1:B78">
+  <sortState ref="B1:B78">
     <sortCondition ref="B1:B78"/>
   </sortState>
   <hyperlinks>
@@ -17145,7 +17134,7 @@
       <c r="D52" s="44"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G22:G36">
+  <sortState ref="G22:G36">
     <sortCondition ref="G22"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18028,7 +18017,7 @@
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -18190,23 +18179,23 @@
         <v>2020</v>
       </c>
       <c r="D4" s="80">
-        <f t="shared" ref="D4:D10" si="0">AVERAGE(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
+        <f t="shared" ref="D4:D9" si="0">AVERAGE(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
         <v>2003.75</v>
       </c>
       <c r="E4" s="43">
-        <f t="shared" ref="E4:E10" si="1">MEDIAN(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
+        <f t="shared" ref="E4:E9" si="1">MEDIAN(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
         <v>2003.75</v>
       </c>
       <c r="F4" s="43">
-        <f t="shared" ref="F4:F10" si="2">MIN(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
+        <f t="shared" ref="F4:F9" si="2">MIN(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
         <v>7.5</v>
       </c>
       <c r="G4" s="43">
-        <f t="shared" ref="G4:G10" si="3">MAX(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
+        <f t="shared" ref="G4:G9" si="3">MAX(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4)</f>
         <v>4000</v>
       </c>
       <c r="H4" s="39">
-        <f t="shared" ref="H4:H10" si="4">COUNT(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4,AS4)</f>
+        <f t="shared" ref="H4:H9" si="4">COUNT(I4,J4,K4,L4,M4,N4,O4,P4,Q4,R4,S4,T4,U4,Y4,AC4,AG4,AK4,AO4,AS4)</f>
         <v>2</v>
       </c>
       <c r="I4" s="61"/>
@@ -18228,7 +18217,7 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>111</v>
@@ -18238,42 +18227,46 @@
       </c>
       <c r="D5" s="80">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>138.10166666666666</v>
       </c>
       <c r="E5" s="43">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>72.38</v>
       </c>
       <c r="F5" s="43">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>5.9250000000000007</v>
       </c>
       <c r="G5" s="43">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>336</v>
       </c>
       <c r="H5" s="39">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
+      <c r="J5" s="55">
+        <v>336</v>
+      </c>
       <c r="K5" s="61"/>
-      <c r="L5" s="61"/>
+      <c r="L5" s="55"/>
       <c r="M5" s="61"/>
-      <c r="N5" s="61"/>
-      <c r="O5" s="61"/>
-      <c r="P5" s="61"/>
+      <c r="N5" s="55">
+        <v>72.38</v>
+      </c>
+      <c r="O5" s="61">
+        <v>5.9250000000000007</v>
+      </c>
+      <c r="P5" s="55"/>
       <c r="Q5" s="61"/>
-      <c r="R5" s="61"/>
-      <c r="S5" s="61">
-        <v>9</v>
-      </c>
-      <c r="T5" s="88"/>
+      <c r="R5" s="55"/>
+      <c r="S5" s="61"/>
+      <c r="T5" s="74"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>111</v>
@@ -18283,46 +18276,42 @@
       </c>
       <c r="D6" s="80">
         <f t="shared" si="0"/>
-        <v>138.10166666666666</v>
+        <v>1.3</v>
       </c>
       <c r="E6" s="43">
         <f t="shared" si="1"/>
-        <v>72.38</v>
+        <v>1.3</v>
       </c>
       <c r="F6" s="43">
         <f t="shared" si="2"/>
-        <v>5.9250000000000007</v>
+        <v>1.3</v>
       </c>
       <c r="G6" s="43">
         <f t="shared" si="3"/>
-        <v>336</v>
+        <v>1.3</v>
       </c>
       <c r="H6" s="39">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I6" s="61"/>
-      <c r="J6" s="55">
-        <v>336</v>
-      </c>
+      <c r="J6" s="61"/>
       <c r="K6" s="61"/>
-      <c r="L6" s="55"/>
+      <c r="L6" s="61"/>
       <c r="M6" s="61"/>
-      <c r="N6" s="55">
-        <v>72.38</v>
-      </c>
+      <c r="N6" s="61"/>
       <c r="O6" s="61">
-        <v>5.9250000000000007</v>
-      </c>
-      <c r="P6" s="55"/>
+        <v>1.3</v>
+      </c>
+      <c r="P6" s="61"/>
       <c r="Q6" s="61"/>
-      <c r="R6" s="55"/>
+      <c r="R6" s="61"/>
       <c r="S6" s="61"/>
-      <c r="T6" s="74"/>
+      <c r="T6" s="88"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B7" s="30" t="s">
         <v>111</v>
@@ -18332,42 +18321,62 @@
       </c>
       <c r="D7" s="80">
         <f t="shared" si="0"/>
-        <v>1.3</v>
+        <v>38.839469696969701</v>
       </c>
       <c r="E7" s="43">
         <f t="shared" si="1"/>
-        <v>1.3</v>
+        <v>24</v>
       </c>
       <c r="F7" s="43">
         <f t="shared" si="2"/>
-        <v>1.3</v>
+        <v>5.17</v>
       </c>
       <c r="G7" s="43">
         <f t="shared" si="3"/>
-        <v>1.3</v>
+        <v>80</v>
       </c>
       <c r="H7" s="39">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
-      <c r="L7" s="61"/>
-      <c r="M7" s="61"/>
-      <c r="N7" s="61"/>
+        <v>11</v>
+      </c>
+      <c r="I7" s="61">
+        <v>80</v>
+      </c>
+      <c r="J7" s="61">
+        <v>24</v>
+      </c>
+      <c r="K7" s="61">
+        <v>54.812499999999993</v>
+      </c>
+      <c r="L7" s="61">
+        <v>80</v>
+      </c>
+      <c r="M7" s="61">
+        <v>49.666666666666664</v>
+      </c>
+      <c r="N7" s="61">
+        <v>5.17</v>
+      </c>
       <c r="O7" s="61">
-        <v>1.3</v>
-      </c>
-      <c r="P7" s="61"/>
-      <c r="Q7" s="61"/>
-      <c r="R7" s="61"/>
-      <c r="S7" s="61"/>
+        <v>63.584999999999994</v>
+      </c>
+      <c r="P7" s="61">
+        <v>10</v>
+      </c>
+      <c r="Q7" s="61">
+        <v>20</v>
+      </c>
+      <c r="R7" s="61">
+        <v>20</v>
+      </c>
+      <c r="S7" s="61">
+        <v>20</v>
+      </c>
       <c r="T7" s="88"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="B8" s="30" t="s">
         <v>111</v>
@@ -18377,62 +18386,44 @@
       </c>
       <c r="D8" s="80">
         <f t="shared" si="0"/>
-        <v>38.839469696969701</v>
+        <v>350.54</v>
       </c>
       <c r="E8" s="43">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>350.54</v>
       </c>
       <c r="F8" s="43">
         <f t="shared" si="2"/>
-        <v>5.17</v>
+        <v>124.08</v>
       </c>
       <c r="G8" s="43">
         <f t="shared" si="3"/>
-        <v>80</v>
+        <v>577</v>
       </c>
       <c r="H8" s="39">
         <f t="shared" si="4"/>
-        <v>11</v>
-      </c>
-      <c r="I8" s="61">
-        <v>80</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="I8" s="61"/>
       <c r="J8" s="61">
-        <v>24</v>
-      </c>
-      <c r="K8" s="61">
-        <v>54.812499999999993</v>
-      </c>
-      <c r="L8" s="61">
-        <v>80</v>
-      </c>
-      <c r="M8" s="61">
-        <v>49.666666666666664</v>
-      </c>
+        <v>577</v>
+      </c>
+      <c r="K8" s="61"/>
+      <c r="L8" s="61"/>
+      <c r="M8" s="61"/>
       <c r="N8" s="61">
-        <v>5.17</v>
-      </c>
-      <c r="O8" s="61">
-        <v>63.584999999999994</v>
-      </c>
-      <c r="P8" s="61">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="61">
-        <v>20</v>
-      </c>
-      <c r="R8" s="61">
-        <v>20</v>
-      </c>
-      <c r="S8" s="61">
-        <v>20</v>
-      </c>
+        <v>124.08</v>
+      </c>
+      <c r="O8" s="61"/>
+      <c r="P8" s="61"/>
+      <c r="Q8" s="61"/>
+      <c r="R8" s="61"/>
+      <c r="S8" s="61"/>
       <c r="T8" s="88"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>57</v>
       </c>
       <c r="B9" s="30" t="s">
         <v>111</v>
@@ -18442,94 +18433,88 @@
       </c>
       <c r="D9" s="80">
         <f t="shared" si="0"/>
-        <v>350.54</v>
+        <v>16.734999999999999</v>
       </c>
       <c r="E9" s="43">
         <f t="shared" si="1"/>
-        <v>350.54</v>
+        <v>16.734999999999999</v>
       </c>
       <c r="F9" s="43">
         <f t="shared" si="2"/>
-        <v>124.08</v>
+        <v>16.734999999999999</v>
       </c>
       <c r="G9" s="43">
         <f t="shared" si="3"/>
-        <v>577</v>
+        <v>16.734999999999999</v>
       </c>
       <c r="H9" s="39">
         <f t="shared" si="4"/>
-        <v>2</v>
-      </c>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61">
-        <v>577</v>
-      </c>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="61"/>
-      <c r="N9" s="61">
-        <v>124.08</v>
-      </c>
-      <c r="O9" s="61"/>
-      <c r="P9" s="61"/>
-      <c r="Q9" s="61"/>
-      <c r="R9" s="61"/>
-      <c r="S9" s="61"/>
-      <c r="T9" s="88"/>
+        <v>1</v>
+      </c>
+      <c r="I9" s="55"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+      <c r="M9" s="55"/>
+      <c r="N9" s="55"/>
+      <c r="O9" s="55">
+        <v>16.734999999999999</v>
+      </c>
+      <c r="P9" s="55"/>
+      <c r="Q9" s="55"/>
+      <c r="R9" s="55"/>
+      <c r="S9" s="55"/>
+      <c r="T9" s="74"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="30">
-        <v>2020</v>
-      </c>
-      <c r="D10" s="80">
-        <f t="shared" si="0"/>
-        <v>16.734999999999999</v>
-      </c>
-      <c r="E10" s="43">
-        <f t="shared" si="1"/>
-        <v>16.734999999999999</v>
-      </c>
-      <c r="F10" s="43">
-        <f t="shared" si="2"/>
-        <v>16.734999999999999</v>
-      </c>
-      <c r="G10" s="43">
-        <f t="shared" si="3"/>
-        <v>16.734999999999999</v>
-      </c>
-      <c r="H10" s="39">
-        <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="39"/>
       <c r="I10" s="55"/>
       <c r="J10" s="55"/>
       <c r="K10" s="55"/>
       <c r="L10" s="55"/>
       <c r="M10" s="55"/>
       <c r="N10" s="55"/>
-      <c r="O10" s="55">
-        <v>16.734999999999999</v>
-      </c>
+      <c r="O10" s="55"/>
       <c r="P10" s="55"/>
       <c r="Q10" s="55"/>
       <c r="R10" s="55"/>
       <c r="S10" s="55"/>
       <c r="T10" s="74"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="80"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="39"/>
+    <row r="11" spans="1:20" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="86" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="71" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="71">
+        <v>2050</v>
+      </c>
+      <c r="D11" s="81">
+        <f>AVERAGE(F11:G11)</f>
+        <v>3.085</v>
+      </c>
+      <c r="E11" s="72">
+        <f>AVERAGE(F11:G11)</f>
+        <v>3.085</v>
+      </c>
+      <c r="F11" s="72">
+        <v>1</v>
+      </c>
+      <c r="G11" s="72">
+        <f>F7</f>
+        <v>5.17</v>
+      </c>
+      <c r="H11" s="85" t="s">
+        <v>222</v>
+      </c>
       <c r="I11" s="55"/>
       <c r="J11" s="55"/>
       <c r="K11" s="55"/>
@@ -18543,72 +18528,31 @@
       <c r="S11" s="55"/>
       <c r="T11" s="74"/>
     </row>
-    <row r="12" spans="1:20" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="86" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="71" t="s">
-        <v>111</v>
-      </c>
-      <c r="C12" s="71">
-        <v>2050</v>
-      </c>
-      <c r="D12" s="81">
-        <f>AVERAGE(F12:G12)</f>
-        <v>3.085</v>
-      </c>
-      <c r="E12" s="72">
-        <f>AVERAGE(F12:G12)</f>
-        <v>3.085</v>
-      </c>
-      <c r="F12" s="72">
-        <v>1</v>
-      </c>
-      <c r="G12" s="72">
-        <f>F8</f>
-        <v>5.17</v>
-      </c>
-      <c r="H12" s="85" t="s">
-        <v>222</v>
-      </c>
-      <c r="I12" s="55"/>
-      <c r="J12" s="55"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="55"/>
-      <c r="M12" s="55"/>
-      <c r="N12" s="55"/>
-      <c r="O12" s="55"/>
-      <c r="P12" s="55"/>
-      <c r="Q12" s="55"/>
-      <c r="R12" s="55"/>
-      <c r="S12" s="55"/>
-      <c r="T12" s="74"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="56"/>
-      <c r="J13" s="56"/>
-      <c r="K13" s="56"/>
-      <c r="L13" s="56"/>
-      <c r="M13" s="56"/>
-      <c r="N13" s="56"/>
-      <c r="O13" s="56"/>
-      <c r="P13" s="56"/>
-      <c r="Q13" s="56"/>
-      <c r="R13" s="56"/>
-      <c r="S13" s="56"/>
-      <c r="T13" s="36"/>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A12" s="26"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="56"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="56"/>
+      <c r="M12" s="56"/>
+      <c r="N12" s="56"/>
+      <c r="O12" s="56"/>
+      <c r="P12" s="56"/>
+      <c r="Q12" s="56"/>
+      <c r="R12" s="56"/>
+      <c r="S12" s="56"/>
+      <c r="T12" s="36"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E24:E42">
-    <sortCondition ref="E24"/>
+  <sortState ref="E23:E41">
+    <sortCondition ref="E23"/>
   </sortState>
   <mergeCells count="1">
     <mergeCell ref="D1:H1"/>

</xml_diff>